<commit_message>
Add PDF report generation with ReportLab
</commit_message>
<xml_diff>
--- a/output/kobe_tourism_report.xlsx
+++ b/output/kobe_tourism_report.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +28,24 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +53,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,56 +438,60 @@
   </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>総スポット数</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>平均評価</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>4.14</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>総レビュー数</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>233780</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>人気スポット</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>神戸どうぶつ王国</t>
         </is>
@@ -486,154 +510,160 @@
   </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>エリア</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>スポット数</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>平均評価</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>総レビュー数</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>4.19</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>127351</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>兵庫区</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>4.08</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>5179</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>北区</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>4.04</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>16079</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>垂水区</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>4.22</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>16240</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>東灘区</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>4.13</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>12701</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>灘区</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2" t="n">
         <v>4.24</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>30397</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>長田区</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="2" t="n">
         <v>3.94</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>7019</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>須磨区</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="2" t="n">
         <v>4.22</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>18814</v>
       </c>
     </row>
@@ -650,240 +680,247 @@
   </sheetPr>
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>カテゴリ</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>スポット数</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>平均評価</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>総レビュー数</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>平均Popularity Score</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>公園</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>4.1</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>26550</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>5.51</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>動物園</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>4.4</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>26258</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>8.31</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>博物館</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>4.13</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>37934</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>5.72</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>商業施設</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>3.74</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>10161</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>4.85</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>宗教施設</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>4.27</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>21495</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>5.49</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>展望台</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2" t="n">
         <v>4.28</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>25151</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>7.33</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>植物園</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="2" t="n">
         <v>4.23</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>10846</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>6.81</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>水族館</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="2" t="n">
         <v>4.07</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>11107</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>6.51</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>牧場</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="2" t="n">
         <v>4.2</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
         <v>3491</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="2" t="n">
         <v>6.85</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>観光地</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="2" t="n">
         <v>4.18</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
         <v>50617</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="2" t="n">
         <v>5.51</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>遊園地</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="2" t="n">
         <v>4.15</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
         <v>10170</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="2" t="n">
         <v>5.52</v>
       </c>
     </row>
@@ -900,331 +937,340 @@
   </sheetPr>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>順位</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>スポット名</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>エリア</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>カテゴリ</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>評価</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>レビュー数</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Popularity Score</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>神戸どうぶつ王国</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>動物園</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>4.5</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>16882</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="2" t="n">
         <v>8.76</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>生田神社</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>宗教施設</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>4.3</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="n">
         <v>12145</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="2" t="n">
         <v>8.09</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>神戸布引ハーブ園</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>植物園</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>4.5</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="2" t="n">
         <v>6591</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="2" t="n">
         <v>7.91</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>南京町</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>観光地</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>3.9</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="2" t="n">
         <v>24013</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="2" t="n">
         <v>7.87</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>神戸市立王子動物園</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>灘区</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>動物園</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>4.3</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>9376</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="2" t="n">
         <v>7.87</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>神戸ポートタワー</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>展望台</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>4.2</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="2" t="n">
         <v>11457</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="2" t="n">
         <v>7.85</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>掬星台</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>灘区</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>展望台</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>4.5</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="2" t="n">
         <v>4554</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="2" t="n">
         <v>7.58</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>明石海峡大橋</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>垂水区</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>観光地</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="2" t="n">
         <v>3213</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="2" t="n">
         <v>7.43</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>兵庫県立美術館</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>博物館</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="2" t="n">
         <v>4.2</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="2" t="n">
         <v>6596</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="2" t="n">
         <v>7.39</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>BE KOBE モニュメント (メリケンパーク)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>中央区</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>観光地</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="2" t="n">
         <v>4.4</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="2" t="n">
         <v>4305</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="2" t="n">
         <v>7.36</v>
       </c>
     </row>

</xml_diff>